<commit_message>
Script d'extraction sans perte et guide ; PBC : exports .xls du Grenier lisibles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_PBC_complete_pointee_20261018.xlsx
+++ b/FPPN_PBC_complete_pointee_20261018.xlsx
@@ -207,7 +207,7 @@
     <t xml:space="preserve">Prêts aux mutualistes (« Le Grenier du Policier ») au 31/12/2025 et au 31/08/2026 : encours par emprunteur, échéancier de remboursement, montants impayés et leur ancienneté.</t>
   </si>
   <si>
-    <t xml:space="preserve">Reçu au format PDF : balance âgée au 31/12/2025 et au 31/08/2026 (global, CRF, CRO, CRS), avec encours, dates d'échéance et montant des échéances par emprunteur. Les versions .xls sont illisibles. Montants impayés et ancienneté : à confirmer à la lecture des PDF. Reçu en plus : balances âgées fin 2021 à fin 2024, production annuelle 2021 à 2025, politique de crédit du 17/07/2021 (.doc). Rien pour 2020.</t>
+    <t xml:space="preserve">Reçu au format PDF et .xls : balance âgée au 31/12/2025 et au 31/08/2026 (global, CRF, CRO, CRS), avec encours, dates d'échéance et montant des échéances par emprunteur. Les mêmes données existent en .xls : ce sont des exports au format page web, lisibles, mais sans la lettre-clé du mécano. Montants impayés et ancienneté : à confirmer à la lecture des PDF. Reçu en plus : balances âgées fin 2021 à fin 2024, production annuelle 2021 à 2025, politique de crédit du 17/07/2021 (.doc). Rien pour 2020.</t>
   </si>
   <si>
     <t xml:space="preserve">Cotisations retenues par l'État et non reversées au FPPN : montant par année, montants recouvrés, échéancier ou accord de recouvrement.</t>
@@ -2568,10 +2568,10 @@
     <t xml:space="preserve">Grenier : 70 fichiers .xls (BalanceAgee, production_de_la_periode)</t>
   </si>
   <si>
-    <t xml:space="preserve">Format non reconnu (export du logiciel). Les PDF équivalents sont lisibles.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renvoyer en .xlsx ou .csv, au moins les balances âgées au 31/12/2020 à 31/12/2025 et au 31/08/2026.</t>
+    <t xml:space="preserve">Ce sont des exports au format page web (logiciel Zenith Technology), et non de vrais fichiers Excel : ils sont lisibles. Contrôle sur la balance âgée CRS au 31/08/2026 : mêmes montants, dates et totaux que le PDF. Seule différence : le mécano perd sa lettre-clé (321100C devient 321100).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aucun renvoi nécessaire. Demander si possible un export qui conserve la lettre-clé du mécano.</t>
   </si>
   <si>
     <t xml:space="preserve">Grenier : balances âgées 2026</t>
@@ -4164,7 +4164,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="117.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="18" t="n">
         <f aca="false">+B40+1</f>
         <v>21</v>
@@ -29920,7 +29920,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="30" t="n">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
Rapport actuariel et statistique (rapport d'étape au 15/10/2026), classeur des calculs, note interne, PBC mise à jour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_PBC_complete_pointee_20261018.xlsx
+++ b/FPPN_PBC_complete_pointee_20261018.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6660" uniqueCount="868">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6666" uniqueCount="874">
   <si>
     <t xml:space="preserve">AUDIT DU FPPN 2020 – 31 AOÛT 2026 : VOLET ACTUARIEL</t>
   </si>
@@ -120,7 +120,7 @@
     <t xml:space="preserve">Détail des provisions inscrites au bilan, par nature et par garantie, au 31/12/2019, 31/12/2020, 31/12/2021, 31/12/2022, 31/12/2023, 31/12/2024, 31/12/2025 et 31/08/2026, avec la note ou le fichier de calcul de chaque provision.</t>
   </si>
   <si>
-    <t xml:space="preserve">Reçu : balances et grands livres (comptes et tiers), aux dates 31/12/2020, 31/12/2021, 31/12/2022, 31/12/2023, 31/12/2024, 31/12/2025, et 31/08/2026 en impression provisoire. Ils donnent les soldes, pas le détail ni le calcul des provisions. Manque : situation au 31/12/2019 ; écritures de janvier à août 2020 (les fichiers 2020 couvrent le 01/09/2020 au 31/12/2020) ; détail par nature et par garantie et note de calcul, à chacune des 8 dates.</t>
+    <t xml:space="preserve">Reçu : balances et grands livres (comptes et tiers), aux dates 31/12/2020, 31/12/2021, 31/12/2022, 31/12/2023, 31/12/2024, 31/12/2025, et 31/08/2026 en impression provisoire. Ils donnent les soldes, pas le détail ni le calcul des provisions. Les balances 2020 donnent les totaux de l'année entière (colonne de cumul au 31/08/2020). Manque : situation au 31/12/2019 ; détail des écritures de janvier à août 2020 ; détail par nature et par garantie et note de calcul, à chacune des 8 dates.</t>
   </si>
   <si>
     <t xml:space="preserve">Tout rapport actuariel, étude technique ou note de calcul des engagements envers les mutualistes existant, quelle que soit sa date.</t>
@@ -2469,7 +2469,7 @@
     <t xml:space="preserve">Comptabilité de janvier à août 2020</t>
   </si>
   <si>
-    <t xml:space="preserve">Les balances et grands livres 2020 couvrent le 01/09/2020 au 31/12/2020. Le dossier comptable change de nom au 01/01/2021 (« FPPN PCMS 2021 »).</t>
+    <t xml:space="preserve">Les balances 2020 donnent les totaux de l'année entière (cumul au 31/08/2020), mais le détail des écritures commence au 01/09/2020. Le dossier comptable change de nom au 01/01/2021 (« FPPN PCMS 2021 »).</t>
   </si>
   <si>
     <t xml:space="preserve">Transmettre les balances et grands livres du 01/01/2020 au 31/08/2020, la balance au 31/12/2019 et les états financiers 2019 à 2025.</t>
@@ -2505,7 +2505,7 @@
     <t xml:space="preserve">SOLDE\EFFECTIF POLICE (MALADIE)\2024\122024_effectif_police_936_DECEMBRE 2024.xlsx et SOLDE\ALLOCATION DECES\2024\FPPN_ALLOC_DECES_8Z6_DECEMBRE_2024.xlsx</t>
   </si>
   <si>
-    <t xml:space="preserve">Les deux fichiers sont endommagés et identiques octet pour octet : un même fichier a été copié sous deux noms.</t>
+    <t xml:space="preserve">Les deux fichiers sont vides (0 octet) et identiques : aucune donnée pour décembre 2024.</t>
   </si>
   <si>
     <t xml:space="preserve">Renvoyer les deux fichiers de décembre 2024.</t>
@@ -2592,13 +2592,13 @@
     <t xml:space="preserve">Renvoyer en .docx ou .pdf, et confirmer qu'il s'agit de la version en vigueur.</t>
   </si>
   <si>
-    <t xml:space="preserve">DAFC : 5 fichiers endommagés (balance des tiers 2021 et 2025 .xlsx ; grand livre des comptes 2022 et 2025 .pdf ; grand livre des tiers 2023 .xlsx)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L'autre format (PDF ou Excel) est lisible pour chacun : pas de manque de contenu.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renvoyer les versions Excel si possible.</t>
+    <t xml:space="preserve">DAFC : 7 fichiers Excel endommagés (balances des tiers 2021 et 2025 ; grands livres des comptes 2021, 2022, 2024 ; grands livres des tiers 2023 et 2025) et 2 PDF endommagés (grands livres des comptes 2022 et 2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les PDF équivalents sont lisibles, sauf le grand livre des comptes 2022 (417 pages récupérées sur 657). Tous les fichiers endommagés viennent du même dossier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refaire l'export depuis Sage des grands livres 2021 à 2025 et des balances des tiers 2021 et 2025 ; préciser comment les fichiers ont été copiés.</t>
   </si>
   <si>
     <t xml:space="preserve">DAFC : intitulés erronés</t>
@@ -2635,6 +2635,24 @@
   </si>
   <si>
     <t xml:space="preserve">Aucune, pour information.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEDOC 8Z7 : retours de février et avril 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les deux fichiers ne contiennent que « aucune ligne sélectionnée ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmer qu'aucun précompte MEDOC n'a été fait ces deux mois, ou transmettre les bons fichiers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identifiants « 183FPPN » (34 identifiants, 224 lignes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichiers aller PEP 998 et Grenier 9X4 de 2025 et 2026 : identifiant interne à la place du mécano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préciser qui sont ces personnes (agents du FPPN ?) et donner leur mécano.</t>
   </si>
 </sst>
 </file>
@@ -29733,7 +29751,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:E24"/>
+  <dimension ref="B2:E26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -29766,7 +29784,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="30" t="n">
         <v>1</v>
       </c>
@@ -29962,7 +29980,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="30" t="n">
         <v>15</v>
       </c>
@@ -30030,6 +30048,34 @@
       </c>
       <c r="E24" s="31" t="s">
         <v>867</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="30" t="n">
+        <v>20</v>
+      </c>
+      <c r="C25" s="31" t="s">
+        <v>868</v>
+      </c>
+      <c r="D25" s="31" t="s">
+        <v>869</v>
+      </c>
+      <c r="E25" s="31" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="30" t="n">
+        <v>21</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>871</v>
+      </c>
+      <c r="D26" s="31" t="s">
+        <v>872</v>
+      </c>
+      <c r="E26" s="31" t="s">
+        <v>873</v>
       </c>
     </row>
   </sheetData>

</xml_diff>